<commit_message>
data: RangeSayacv3_yeni_taslak revize edildi
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/RangeSayacv3_yeni_taslak.xlsx
+++ b/RangeSayacv3_yeni_taslak.xlsx
@@ -8,14 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\kaank\Downloads\IpekyolRangeSayac\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D9A82489-966E-47E4-87F0-80C47D10CB63}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4482AD1A-E3D5-4681-92EF-EA865B7B0D40}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="19090" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sayfa1" sheetId="1" r:id="rId1"/>
     <sheet name="Sayfa2" sheetId="3" r:id="rId2"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Sayfa1!$A$1:$I$827</definedName>
+  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -42,7 +45,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3527" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3647" uniqueCount="176">
   <si>
     <t>Tema Adı</t>
   </si>
@@ -565,12 +568,18 @@
   <si>
     <t>TRAVEL SET</t>
   </si>
+  <si>
+    <t>Mono-Weekend Edit 2</t>
+  </si>
+  <si>
+    <t>Jean SP1</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="5" x14ac:knownFonts="1">
+  <fonts count="6" x14ac:knownFonts="1">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -610,6 +619,12 @@
       <name val="Arial"/>
       <family val="2"/>
       <charset val="162"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="9">
@@ -1065,7 +1080,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I827"/>
+  <dimension ref="A1:I857"/>
   <sheetFormatPr defaultRowHeight="15.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="19.125" customWidth="1"/>
@@ -1695,7 +1710,7 @@
         <v>49</v>
       </c>
       <c r="I21" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22" spans="1:9" x14ac:dyDescent="0.25">
@@ -1726,7 +1741,7 @@
         <v>13</v>
       </c>
       <c r="I22" s="1">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="23" spans="1:9" x14ac:dyDescent="0.25">
@@ -1786,7 +1801,7 @@
         <v>17</v>
       </c>
       <c r="I24" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="25" spans="1:9" x14ac:dyDescent="0.25">
@@ -1817,7 +1832,7 @@
         <v>14</v>
       </c>
       <c r="I25" s="1">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="26" spans="1:9" x14ac:dyDescent="0.25">
@@ -1847,9 +1862,7 @@
         <f>VLOOKUP(G26,Sayfa2!M:N,2,0)</f>
         <v>52</v>
       </c>
-      <c r="I26" s="1">
-        <v>1</v>
-      </c>
+      <c r="I26" s="1"/>
     </row>
     <row r="27" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
@@ -1909,7 +1922,9 @@
         <f>VLOOKUP(G28,Sayfa2!M:N,2,0)</f>
         <v>22</v>
       </c>
-      <c r="I28" s="1"/>
+      <c r="I28" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="29" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
@@ -1939,7 +1954,7 @@
         <v>23</v>
       </c>
       <c r="I29" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:9" x14ac:dyDescent="0.25">
@@ -1998,7 +2013,9 @@
         <f>VLOOKUP(G31,Sayfa2!M:N,2,0)</f>
         <v>50</v>
       </c>
-      <c r="I31" s="1"/>
+      <c r="I31" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="32" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
@@ -25943,7 +25960,852 @@
         <v>1</v>
       </c>
     </row>
+    <row r="828" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A828" t="s">
+        <v>40</v>
+      </c>
+      <c r="B828">
+        <v>4</v>
+      </c>
+      <c r="C828">
+        <v>10</v>
+      </c>
+      <c r="D828" t="s">
+        <v>37</v>
+      </c>
+      <c r="E828" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F828">
+        <v>1327</v>
+      </c>
+      <c r="G828" t="s">
+        <v>4</v>
+      </c>
+      <c r="H828">
+        <f>VLOOKUP(G828,Sayfa2!M:N,2,0)</f>
+        <v>21</v>
+      </c>
+      <c r="I828" s="1"/>
+    </row>
+    <row r="829" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A829" t="s">
+        <v>40</v>
+      </c>
+      <c r="B829">
+        <v>4</v>
+      </c>
+      <c r="C829">
+        <v>10</v>
+      </c>
+      <c r="D829" t="s">
+        <v>37</v>
+      </c>
+      <c r="E829" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F829">
+        <v>1327</v>
+      </c>
+      <c r="G829" t="s">
+        <v>5</v>
+      </c>
+      <c r="H829">
+        <f>VLOOKUP(G829,Sayfa2!M:N,2,0)</f>
+        <v>19</v>
+      </c>
+      <c r="I829" s="1"/>
+    </row>
+    <row r="830" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A830" t="s">
+        <v>40</v>
+      </c>
+      <c r="B830">
+        <v>4</v>
+      </c>
+      <c r="C830">
+        <v>10</v>
+      </c>
+      <c r="D830" t="s">
+        <v>37</v>
+      </c>
+      <c r="E830" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F830">
+        <v>1327</v>
+      </c>
+      <c r="G830" t="s">
+        <v>6</v>
+      </c>
+      <c r="H830">
+        <f>VLOOKUP(G830,Sayfa2!M:N,2,0)</f>
+        <v>20</v>
+      </c>
+      <c r="I830" s="1"/>
+    </row>
+    <row r="831" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A831" t="s">
+        <v>40</v>
+      </c>
+      <c r="B831">
+        <v>4</v>
+      </c>
+      <c r="C831">
+        <v>10</v>
+      </c>
+      <c r="D831" t="s">
+        <v>37</v>
+      </c>
+      <c r="E831" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F831">
+        <v>1327</v>
+      </c>
+      <c r="G831" t="s">
+        <v>7</v>
+      </c>
+      <c r="H831">
+        <f>VLOOKUP(G831,Sayfa2!M:N,2,0)</f>
+        <v>12</v>
+      </c>
+      <c r="I831" s="1"/>
+    </row>
+    <row r="832" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A832" t="s">
+        <v>40</v>
+      </c>
+      <c r="B832">
+        <v>4</v>
+      </c>
+      <c r="C832">
+        <v>10</v>
+      </c>
+      <c r="D832" t="s">
+        <v>37</v>
+      </c>
+      <c r="E832" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F832">
+        <v>1327</v>
+      </c>
+      <c r="G832" t="s">
+        <v>8</v>
+      </c>
+      <c r="H832">
+        <f>VLOOKUP(G832,Sayfa2!M:N,2,0)</f>
+        <v>49</v>
+      </c>
+      <c r="I832" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="833" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A833" t="s">
+        <v>40</v>
+      </c>
+      <c r="B833">
+        <v>4</v>
+      </c>
+      <c r="C833">
+        <v>10</v>
+      </c>
+      <c r="D833" t="s">
+        <v>37</v>
+      </c>
+      <c r="E833" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F833">
+        <v>1327</v>
+      </c>
+      <c r="G833" t="s">
+        <v>9</v>
+      </c>
+      <c r="H833">
+        <f>VLOOKUP(G833,Sayfa2!M:N,2,0)</f>
+        <v>13</v>
+      </c>
+      <c r="I833" s="1"/>
+    </row>
+    <row r="834" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A834" t="s">
+        <v>40</v>
+      </c>
+      <c r="B834">
+        <v>4</v>
+      </c>
+      <c r="C834">
+        <v>10</v>
+      </c>
+      <c r="D834" t="s">
+        <v>37</v>
+      </c>
+      <c r="E834" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F834">
+        <v>1327</v>
+      </c>
+      <c r="G834" t="s">
+        <v>10</v>
+      </c>
+      <c r="H834">
+        <f>VLOOKUP(G834,Sayfa2!M:N,2,0)</f>
+        <v>16</v>
+      </c>
+      <c r="I834" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="835" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A835" t="s">
+        <v>40</v>
+      </c>
+      <c r="B835">
+        <v>4</v>
+      </c>
+      <c r="C835">
+        <v>10</v>
+      </c>
+      <c r="D835" t="s">
+        <v>37</v>
+      </c>
+      <c r="E835" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F835">
+        <v>1327</v>
+      </c>
+      <c r="G835" t="s">
+        <v>11</v>
+      </c>
+      <c r="H835">
+        <f>VLOOKUP(G835,Sayfa2!M:N,2,0)</f>
+        <v>17</v>
+      </c>
+      <c r="I835" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="836" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A836" t="s">
+        <v>40</v>
+      </c>
+      <c r="B836">
+        <v>4</v>
+      </c>
+      <c r="C836">
+        <v>10</v>
+      </c>
+      <c r="D836" t="s">
+        <v>37</v>
+      </c>
+      <c r="E836" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F836">
+        <v>1327</v>
+      </c>
+      <c r="G836" t="s">
+        <v>12</v>
+      </c>
+      <c r="H836">
+        <f>VLOOKUP(G836,Sayfa2!M:N,2,0)</f>
+        <v>14</v>
+      </c>
+      <c r="I836" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="837" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A837" t="s">
+        <v>40</v>
+      </c>
+      <c r="B837">
+        <v>4</v>
+      </c>
+      <c r="C837">
+        <v>10</v>
+      </c>
+      <c r="D837" t="s">
+        <v>37</v>
+      </c>
+      <c r="E837" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F837">
+        <v>1327</v>
+      </c>
+      <c r="G837" t="s">
+        <v>13</v>
+      </c>
+      <c r="H837">
+        <f>VLOOKUP(G837,Sayfa2!M:N,2,0)</f>
+        <v>52</v>
+      </c>
+      <c r="I837" s="1"/>
+    </row>
+    <row r="838" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A838" t="s">
+        <v>40</v>
+      </c>
+      <c r="B838">
+        <v>4</v>
+      </c>
+      <c r="C838">
+        <v>10</v>
+      </c>
+      <c r="D838" t="s">
+        <v>37</v>
+      </c>
+      <c r="E838" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F838">
+        <v>1327</v>
+      </c>
+      <c r="G838" t="s">
+        <v>14</v>
+      </c>
+      <c r="H838">
+        <f>VLOOKUP(G838,Sayfa2!M:N,2,0)</f>
+        <v>27</v>
+      </c>
+      <c r="I838" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="839" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A839" t="s">
+        <v>40</v>
+      </c>
+      <c r="B839">
+        <v>4</v>
+      </c>
+      <c r="C839">
+        <v>10</v>
+      </c>
+      <c r="D839" t="s">
+        <v>37</v>
+      </c>
+      <c r="E839" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F839">
+        <v>1327</v>
+      </c>
+      <c r="G839" t="s">
+        <v>15</v>
+      </c>
+      <c r="H839">
+        <f>VLOOKUP(G839,Sayfa2!M:N,2,0)</f>
+        <v>22</v>
+      </c>
+      <c r="I839" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="840" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A840" t="s">
+        <v>40</v>
+      </c>
+      <c r="B840">
+        <v>4</v>
+      </c>
+      <c r="C840">
+        <v>10</v>
+      </c>
+      <c r="D840" t="s">
+        <v>37</v>
+      </c>
+      <c r="E840" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F840">
+        <v>1327</v>
+      </c>
+      <c r="G840" t="s">
+        <v>16</v>
+      </c>
+      <c r="H840">
+        <f>VLOOKUP(G840,Sayfa2!M:N,2,0)</f>
+        <v>23</v>
+      </c>
+      <c r="I840" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="841" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A841" t="s">
+        <v>40</v>
+      </c>
+      <c r="B841">
+        <v>4</v>
+      </c>
+      <c r="C841">
+        <v>10</v>
+      </c>
+      <c r="D841" t="s">
+        <v>37</v>
+      </c>
+      <c r="E841" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F841">
+        <v>1327</v>
+      </c>
+      <c r="G841" t="s">
+        <v>17</v>
+      </c>
+      <c r="H841">
+        <f>VLOOKUP(G841,Sayfa2!M:N,2,0)</f>
+        <v>25</v>
+      </c>
+      <c r="I841" s="1"/>
+    </row>
+    <row r="842" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A842" t="s">
+        <v>40</v>
+      </c>
+      <c r="B842">
+        <v>4</v>
+      </c>
+      <c r="C842">
+        <v>10</v>
+      </c>
+      <c r="D842" t="s">
+        <v>37</v>
+      </c>
+      <c r="E842" s="2" t="s">
+        <v>174</v>
+      </c>
+      <c r="F842">
+        <v>1327</v>
+      </c>
+      <c r="G842" t="s">
+        <v>18</v>
+      </c>
+      <c r="H842">
+        <f>VLOOKUP(G842,Sayfa2!M:N,2,0)</f>
+        <v>50</v>
+      </c>
+      <c r="I842" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="843" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A843" t="s">
+        <v>40</v>
+      </c>
+      <c r="B843">
+        <v>4</v>
+      </c>
+      <c r="C843">
+        <v>10</v>
+      </c>
+      <c r="D843" t="s">
+        <v>37</v>
+      </c>
+      <c r="E843" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F843">
+        <v>1228</v>
+      </c>
+      <c r="G843" t="s">
+        <v>4</v>
+      </c>
+      <c r="H843">
+        <f>VLOOKUP(G843,Sayfa2!M:N,2,0)</f>
+        <v>21</v>
+      </c>
+    </row>
+    <row r="844" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A844" t="s">
+        <v>40</v>
+      </c>
+      <c r="B844">
+        <v>4</v>
+      </c>
+      <c r="C844">
+        <v>10</v>
+      </c>
+      <c r="D844" t="s">
+        <v>37</v>
+      </c>
+      <c r="E844" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F844">
+        <v>1228</v>
+      </c>
+      <c r="G844" t="s">
+        <v>5</v>
+      </c>
+      <c r="H844">
+        <f>VLOOKUP(G844,Sayfa2!M:N,2,0)</f>
+        <v>19</v>
+      </c>
+    </row>
+    <row r="845" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A845" t="s">
+        <v>40</v>
+      </c>
+      <c r="B845">
+        <v>4</v>
+      </c>
+      <c r="C845">
+        <v>10</v>
+      </c>
+      <c r="D845" t="s">
+        <v>37</v>
+      </c>
+      <c r="E845" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F845">
+        <v>1228</v>
+      </c>
+      <c r="G845" t="s">
+        <v>6</v>
+      </c>
+      <c r="H845">
+        <f>VLOOKUP(G845,Sayfa2!M:N,2,0)</f>
+        <v>20</v>
+      </c>
+    </row>
+    <row r="846" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A846" t="s">
+        <v>40</v>
+      </c>
+      <c r="B846">
+        <v>4</v>
+      </c>
+      <c r="C846">
+        <v>10</v>
+      </c>
+      <c r="D846" t="s">
+        <v>37</v>
+      </c>
+      <c r="E846" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F846">
+        <v>1228</v>
+      </c>
+      <c r="G846" t="s">
+        <v>7</v>
+      </c>
+      <c r="H846">
+        <f>VLOOKUP(G846,Sayfa2!M:N,2,0)</f>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="847" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A847" t="s">
+        <v>40</v>
+      </c>
+      <c r="B847">
+        <v>4</v>
+      </c>
+      <c r="C847">
+        <v>10</v>
+      </c>
+      <c r="D847" t="s">
+        <v>37</v>
+      </c>
+      <c r="E847" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F847">
+        <v>1228</v>
+      </c>
+      <c r="G847" t="s">
+        <v>8</v>
+      </c>
+      <c r="H847">
+        <f>VLOOKUP(G847,Sayfa2!M:N,2,0)</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="848" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A848" t="s">
+        <v>40</v>
+      </c>
+      <c r="B848">
+        <v>4</v>
+      </c>
+      <c r="C848">
+        <v>10</v>
+      </c>
+      <c r="D848" t="s">
+        <v>37</v>
+      </c>
+      <c r="E848" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F848">
+        <v>1228</v>
+      </c>
+      <c r="G848" t="s">
+        <v>9</v>
+      </c>
+      <c r="H848">
+        <f>VLOOKUP(G848,Sayfa2!M:N,2,0)</f>
+        <v>13</v>
+      </c>
+      <c r="I848">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="849" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A849" t="s">
+        <v>40</v>
+      </c>
+      <c r="B849">
+        <v>4</v>
+      </c>
+      <c r="C849">
+        <v>10</v>
+      </c>
+      <c r="D849" t="s">
+        <v>37</v>
+      </c>
+      <c r="E849" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F849">
+        <v>1228</v>
+      </c>
+      <c r="G849" t="s">
+        <v>10</v>
+      </c>
+      <c r="H849">
+        <f>VLOOKUP(G849,Sayfa2!M:N,2,0)</f>
+        <v>16</v>
+      </c>
+    </row>
+    <row r="850" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A850" t="s">
+        <v>40</v>
+      </c>
+      <c r="B850">
+        <v>4</v>
+      </c>
+      <c r="C850">
+        <v>10</v>
+      </c>
+      <c r="D850" t="s">
+        <v>37</v>
+      </c>
+      <c r="E850" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F850">
+        <v>1228</v>
+      </c>
+      <c r="G850" t="s">
+        <v>11</v>
+      </c>
+      <c r="H850">
+        <f>VLOOKUP(G850,Sayfa2!M:N,2,0)</f>
+        <v>17</v>
+      </c>
+    </row>
+    <row r="851" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A851" t="s">
+        <v>40</v>
+      </c>
+      <c r="B851">
+        <v>4</v>
+      </c>
+      <c r="C851">
+        <v>10</v>
+      </c>
+      <c r="D851" t="s">
+        <v>37</v>
+      </c>
+      <c r="E851" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F851">
+        <v>1228</v>
+      </c>
+      <c r="G851" t="s">
+        <v>12</v>
+      </c>
+      <c r="H851">
+        <f>VLOOKUP(G851,Sayfa2!M:N,2,0)</f>
+        <v>14</v>
+      </c>
+    </row>
+    <row r="852" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A852" t="s">
+        <v>40</v>
+      </c>
+      <c r="B852">
+        <v>4</v>
+      </c>
+      <c r="C852">
+        <v>10</v>
+      </c>
+      <c r="D852" t="s">
+        <v>37</v>
+      </c>
+      <c r="E852" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F852">
+        <v>1228</v>
+      </c>
+      <c r="G852" t="s">
+        <v>13</v>
+      </c>
+      <c r="H852">
+        <f>VLOOKUP(G852,Sayfa2!M:N,2,0)</f>
+        <v>52</v>
+      </c>
+    </row>
+    <row r="853" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A853" t="s">
+        <v>40</v>
+      </c>
+      <c r="B853">
+        <v>4</v>
+      </c>
+      <c r="C853">
+        <v>10</v>
+      </c>
+      <c r="D853" t="s">
+        <v>37</v>
+      </c>
+      <c r="E853" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F853">
+        <v>1228</v>
+      </c>
+      <c r="G853" t="s">
+        <v>14</v>
+      </c>
+      <c r="H853">
+        <f>VLOOKUP(G853,Sayfa2!M:N,2,0)</f>
+        <v>27</v>
+      </c>
+    </row>
+    <row r="854" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A854" t="s">
+        <v>40</v>
+      </c>
+      <c r="B854">
+        <v>4</v>
+      </c>
+      <c r="C854">
+        <v>10</v>
+      </c>
+      <c r="D854" t="s">
+        <v>37</v>
+      </c>
+      <c r="E854" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F854">
+        <v>1228</v>
+      </c>
+      <c r="G854" t="s">
+        <v>15</v>
+      </c>
+      <c r="H854">
+        <f>VLOOKUP(G854,Sayfa2!M:N,2,0)</f>
+        <v>22</v>
+      </c>
+    </row>
+    <row r="855" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A855" t="s">
+        <v>40</v>
+      </c>
+      <c r="B855">
+        <v>4</v>
+      </c>
+      <c r="C855">
+        <v>10</v>
+      </c>
+      <c r="D855" t="s">
+        <v>37</v>
+      </c>
+      <c r="E855" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F855">
+        <v>1228</v>
+      </c>
+      <c r="G855" t="s">
+        <v>16</v>
+      </c>
+      <c r="H855">
+        <f>VLOOKUP(G855,Sayfa2!M:N,2,0)</f>
+        <v>23</v>
+      </c>
+    </row>
+    <row r="856" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A856" t="s">
+        <v>40</v>
+      </c>
+      <c r="B856">
+        <v>4</v>
+      </c>
+      <c r="C856">
+        <v>10</v>
+      </c>
+      <c r="D856" t="s">
+        <v>37</v>
+      </c>
+      <c r="E856" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F856">
+        <v>1228</v>
+      </c>
+      <c r="G856" t="s">
+        <v>17</v>
+      </c>
+      <c r="H856">
+        <f>VLOOKUP(G856,Sayfa2!M:N,2,0)</f>
+        <v>25</v>
+      </c>
+    </row>
+    <row r="857" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A857" t="s">
+        <v>40</v>
+      </c>
+      <c r="B857">
+        <v>4</v>
+      </c>
+      <c r="C857">
+        <v>10</v>
+      </c>
+      <c r="D857" t="s">
+        <v>37</v>
+      </c>
+      <c r="E857" s="2" t="s">
+        <v>175</v>
+      </c>
+      <c r="F857">
+        <v>1228</v>
+      </c>
+      <c r="G857" t="s">
+        <v>18</v>
+      </c>
+      <c r="H857">
+        <f>VLOOKUP(G857,Sayfa2!M:N,2,0)</f>
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>